<commit_message>
Funcionalidades Tela de Vendas
</commit_message>
<xml_diff>
--- a/quipaesapp/assets/Dados_Api_Quipaes.xlsx
+++ b/quipaesapp/assets/Dados_Api_Quipaes.xlsx
@@ -1,19 +1,39 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30117"/>
   <workbookPr/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{75E73A6D-6130-4904-B196-123C392CCBE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Compras" sheetId="1" r:id="rId5"/>
-    <sheet state="visible" name="Produtos" sheetId="2" r:id="rId6"/>
-    <sheet state="visible" name="Compras_itens" sheetId="3" r:id="rId7"/>
+    <sheet name="Compras" sheetId="1" r:id="rId1"/>
+    <sheet name="Produtos" sheetId="2" r:id="rId2"/>
+    <sheet name="Compras_itens" sheetId="3" r:id="rId3"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="191028"/>
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="83">
   <si>
     <t>id_compra</t>
   </si>
@@ -36,15 +56,24 @@
     <t>valor_entrega</t>
   </si>
   <si>
+    <t>forma_pgto</t>
+  </si>
+  <si>
     <t>2026-11-22 23:45:17.432679</t>
   </si>
   <si>
     <t>Rua Camatei 19, Vila Nivi, SP</t>
   </si>
   <si>
+    <t>Pix</t>
+  </si>
+  <si>
     <t>2026-11-23 03:19:10.184802</t>
   </si>
   <si>
+    <t>Dinheiro</t>
+  </si>
+  <si>
     <t>2026-11-23 03:20:46.817775</t>
   </si>
   <si>
@@ -54,12 +83,18 @@
     <t>2026-11-23 21:55:53.716342</t>
   </si>
   <si>
+    <t>Crédito</t>
+  </si>
+  <si>
     <t>2026-11-23 19:02:13.959203</t>
   </si>
   <si>
     <t>2026-11-23 23:15:40.263170</t>
   </si>
   <si>
+    <t>Débito</t>
+  </si>
+  <si>
     <t>2026-11-23 23:19:32.211238</t>
   </si>
   <si>
@@ -70,6 +105,9 @@
   </si>
   <si>
     <t>Rua dos peidoreiros 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">	</t>
   </si>
   <si>
     <t>2026-11-23 23:23:46.674072</t>
@@ -249,25 +287,27 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="4">
     <font>
-      <sz val="11.0"/>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
     <font>
-      <sz val="11.0"/>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
     </font>
@@ -277,53 +317,49 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+  <cellXfs count="6">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="14" xfId="0" applyFont="1" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -513,27 +549,27 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-  <sheetPr>
-    <pageSetUpPr/>
-  </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:I991"/>
+  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="10.38"/>
-    <col customWidth="1" min="2" max="2" width="25.0"/>
-    <col customWidth="1" min="3" max="3" width="14.0"/>
-    <col customWidth="1" min="4" max="4" width="26.88"/>
-    <col customWidth="1" min="5" max="5" width="14.25"/>
-    <col customWidth="1" min="6" max="6" width="12.0"/>
-    <col customWidth="1" min="7" max="7" width="12.88"/>
-    <col customWidth="1" min="8" max="26" width="8.63"/>
+    <col min="1" max="1" width="10.42578125" customWidth="1"/>
+    <col min="2" max="2" width="25" customWidth="1"/>
+    <col min="3" max="3" width="14" customWidth="1"/>
+    <col min="4" max="4" width="26.85546875" customWidth="1"/>
+    <col min="5" max="5" width="14.28515625" customWidth="1"/>
+    <col min="6" max="6" width="12" customWidth="1"/>
+    <col min="7" max="7" width="12.85546875" customWidth="1"/>
+    <col min="8" max="26" width="8.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:9" ht="29.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -555,500 +591,569 @@
       <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2">
+      <c r="H1" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
       <c r="A2" s="1">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C2" s="1">
-        <v>5.089712689E10</v>
+        <v>50897126890</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E2" s="1">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F2" s="1">
         <v>45.4</v>
       </c>
       <c r="G2" s="1">
-        <v>5.0</v>
-      </c>
-    </row>
-    <row r="3">
+        <v>5</v>
+      </c>
+      <c r="H2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9">
       <c r="A3" s="1">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="B3" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="1">
+        <v>50897126890</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="1">
-        <v>5.089712689E10</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>8</v>
-      </c>
       <c r="E3" s="1">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F3" s="1">
         <v>45.4</v>
       </c>
       <c r="G3" s="1">
-        <v>5.0</v>
-      </c>
-    </row>
-    <row r="4">
+        <v>5</v>
+      </c>
+      <c r="H3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
       <c r="A4" s="1">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C4" s="1">
-        <v>5.089712689E10</v>
+        <v>50897126890</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E4" s="1">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F4" s="1">
         <v>45.4</v>
       </c>
       <c r="G4" s="1">
-        <v>5.0</v>
-      </c>
-    </row>
-    <row r="5">
+        <v>5</v>
+      </c>
+      <c r="H4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
       <c r="A5" s="1">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C5" s="1">
-        <v>5.089712689E10</v>
+        <v>50897126890</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E5" s="1">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F5" s="1">
-        <v>80.4</v>
+        <v>80.400000000000006</v>
       </c>
       <c r="G5" s="1">
-        <v>5.0</v>
-      </c>
-    </row>
-    <row r="6">
+        <v>5</v>
+      </c>
+      <c r="H5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
       <c r="A6" s="1">
-        <v>5.0</v>
+        <v>5</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C6" s="1">
-        <v>5.089712689E10</v>
+        <v>50897126890</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E6" s="1">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F6" s="1">
         <v>45.4</v>
       </c>
       <c r="G6" s="1">
-        <v>5.0</v>
-      </c>
-    </row>
-    <row r="7">
+        <v>5</v>
+      </c>
+      <c r="H6" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9">
       <c r="A7" s="1">
-        <v>6.0</v>
+        <v>6</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="C7" s="1">
-        <v>5.089712689E10</v>
+        <v>50897126890</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E7" s="1">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F7" s="1">
         <v>25.2</v>
       </c>
       <c r="G7" s="1">
-        <v>5.0</v>
-      </c>
-    </row>
-    <row r="8">
+        <v>5</v>
+      </c>
+      <c r="H7" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9">
       <c r="A8" s="1">
-        <v>8.0</v>
+        <v>8</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C8" s="1">
-        <v>5.089712689E10</v>
+        <v>50897126890</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E8" s="1">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F8" s="1">
         <v>31.5</v>
       </c>
       <c r="G8" s="1">
-        <v>5.0</v>
-      </c>
-    </row>
-    <row r="9">
+        <v>5</v>
+      </c>
+      <c r="H8" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9">
       <c r="A9" s="1">
-        <v>10.0</v>
+        <v>10</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="C9" s="1">
-        <v>9.0019154003E10</v>
+        <v>90019154003</v>
       </c>
       <c r="D9" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E9" s="1">
+        <v>2</v>
+      </c>
+      <c r="F9" s="1">
+        <v>10</v>
+      </c>
+      <c r="G9" s="1">
+        <v>5</v>
+      </c>
+      <c r="H9" t="s">
         <v>16</v>
       </c>
-      <c r="E9" s="1">
-        <v>2.0</v>
-      </c>
-      <c r="F9" s="1">
-        <v>10.0</v>
-      </c>
-      <c r="G9" s="1">
-        <v>5.0</v>
-      </c>
-    </row>
-    <row r="10">
+    </row>
+    <row r="10" spans="1:9">
       <c r="A10" s="1">
-        <v>11.0</v>
+        <v>11</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="C10" s="1">
-        <v>3.003003003E10</v>
+        <v>30030030030</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="E10" s="1">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="F10" s="1">
         <v>31.5</v>
       </c>
       <c r="G10" s="1">
-        <v>5.0</v>
-      </c>
-    </row>
-    <row r="11">
+        <v>5</v>
+      </c>
+      <c r="H10" t="s">
+        <v>16</v>
+      </c>
+      <c r="I10" s="5" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9">
       <c r="A11" s="1">
-        <v>12.0</v>
+        <v>12</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="C11" s="1">
-        <v>3.003003003E10</v>
+        <v>30030030030</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="E11" s="1">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="F11" s="1">
         <v>217.5</v>
       </c>
       <c r="G11" s="1">
-        <v>5.0</v>
-      </c>
-    </row>
-    <row r="12" ht="15.75" customHeight="1">
+        <v>5</v>
+      </c>
+      <c r="H11" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="15.75" customHeight="1">
       <c r="A12" s="1">
-        <v>14.0</v>
+        <v>14</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="C12" s="1">
-        <v>5.089712689E10</v>
+        <v>50897126890</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E12" s="1">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="F12" s="1">
         <v>7.5</v>
       </c>
       <c r="G12" s="1">
-        <v>5.0</v>
-      </c>
-    </row>
-    <row r="13" ht="15.75" customHeight="1">
+        <v>5</v>
+      </c>
+      <c r="H12" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" ht="15.75" customHeight="1">
       <c r="A13" s="1">
-        <v>16.0</v>
+        <v>16</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="C13" s="1">
-        <v>9.0472265008E10</v>
+        <v>90472265008</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="E13" s="1">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F13" s="1">
-        <v>95.6999999999999</v>
+        <v>95.699999999999903</v>
       </c>
       <c r="G13" s="1">
-        <v>5.0</v>
-      </c>
-    </row>
-    <row r="14" ht="15.75" customHeight="1">
+        <v>5</v>
+      </c>
+      <c r="H13" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" ht="15.75" customHeight="1">
       <c r="A14" s="1">
-        <v>17.0</v>
+        <v>17</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="C14" s="1">
-        <v>4.6561535839E10</v>
+        <v>46561535839</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="E14" s="1">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F14" s="1">
         <v>45.4</v>
       </c>
       <c r="G14" s="1">
-        <v>5.0</v>
-      </c>
-    </row>
-    <row r="15" ht="15.75" customHeight="1">
+        <v>5</v>
+      </c>
+      <c r="H14" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" ht="15.75" customHeight="1">
       <c r="A15" s="1">
-        <v>18.0</v>
+        <v>18</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="C15" s="1">
-        <v>4.6561535839E10</v>
+        <v>46561535839</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="E15" s="1">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F15" s="1">
         <v>45.4</v>
       </c>
       <c r="G15" s="1">
-        <v>5.0</v>
-      </c>
-    </row>
-    <row r="16" ht="15.75" customHeight="1">
+        <v>5</v>
+      </c>
+      <c r="H15" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" ht="15.75" customHeight="1">
       <c r="A16" s="1">
-        <v>19.0</v>
+        <v>19</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="C16" s="1">
-        <v>4.8648210895E10</v>
+        <v>48648210895</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="E16" s="1">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="F16" s="1">
-        <v>38.3</v>
+        <v>38.299999999999997</v>
       </c>
       <c r="G16" s="1">
-        <v>5.0</v>
-      </c>
-    </row>
-    <row r="17" ht="15.75" customHeight="1">
+        <v>5</v>
+      </c>
+      <c r="H16" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" ht="15.75" customHeight="1">
       <c r="A17" s="1">
-        <v>20.0</v>
+        <v>20</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="E17" s="1">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F17" s="1">
-        <v>65.6</v>
+        <v>65.599999999999994</v>
       </c>
       <c r="G17" s="1">
-        <v>5.0</v>
-      </c>
-    </row>
-    <row r="18" ht="15.75" customHeight="1">
+        <v>5</v>
+      </c>
+      <c r="H17" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" ht="15.75" customHeight="1">
       <c r="A18" s="1">
-        <v>21.0</v>
+        <v>21</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="C18" s="1">
-        <v>9.0019154003E10</v>
+        <v>90019154003</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="E18" s="1">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F18" s="1">
         <v>25.2</v>
       </c>
       <c r="G18" s="1">
-        <v>5.0</v>
-      </c>
-    </row>
-    <row r="19" ht="15.75" customHeight="1">
+        <v>5</v>
+      </c>
+      <c r="H18" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" ht="15.75" customHeight="1">
       <c r="A19" s="1">
-        <v>22.0</v>
+        <v>22</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="C19" s="1">
-        <v>9.0019154003E10</v>
+        <v>90019154003</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="E19" s="1">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F19" s="1">
-        <v>10.0</v>
+        <v>10</v>
       </c>
       <c r="G19" s="1">
-        <v>5.0</v>
-      </c>
-    </row>
-    <row r="20" ht="15.75" customHeight="1">
+        <v>5</v>
+      </c>
+      <c r="H19" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" ht="15.75" customHeight="1">
       <c r="A20" s="1">
-        <v>23.0</v>
+        <v>23</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="E20" s="1">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="F20" s="1">
         <v>41.2</v>
       </c>
       <c r="G20" s="1">
-        <v>5.0</v>
-      </c>
-    </row>
-    <row r="21" ht="15.75" customHeight="1">
+        <v>5</v>
+      </c>
+      <c r="H20" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" ht="15.75" customHeight="1">
       <c r="A21" s="1">
-        <v>24.0</v>
+        <v>24</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="E21" s="1">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F21" s="1">
-        <v>18.0</v>
+        <v>18</v>
       </c>
       <c r="G21" s="1">
-        <v>5.0</v>
-      </c>
-    </row>
-    <row r="22" ht="15.75" customHeight="1">
+        <v>5</v>
+      </c>
+      <c r="H21" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" ht="15.75" customHeight="1">
       <c r="A22" s="1">
-        <v>25.0</v>
+        <v>25</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="C22" s="1">
-        <v>5.089712689E10</v>
+        <v>50897126890</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E22" s="1">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F22" s="1">
         <v>58.9</v>
       </c>
       <c r="G22" s="1">
-        <v>5.0</v>
-      </c>
-    </row>
-    <row r="23" ht="15.75" customHeight="1"/>
-    <row r="24" ht="15.75" customHeight="1"/>
-    <row r="25" ht="15.75" customHeight="1"/>
-    <row r="26" ht="15.75" customHeight="1"/>
-    <row r="27" ht="15.75" customHeight="1"/>
-    <row r="28" ht="15.75" customHeight="1"/>
-    <row r="29" ht="15.75" customHeight="1"/>
-    <row r="30" ht="15.75" customHeight="1"/>
-    <row r="31" ht="15.75" customHeight="1"/>
-    <row r="32" ht="15.75" customHeight="1"/>
+        <v>5</v>
+      </c>
+      <c r="H22" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" ht="15.75" customHeight="1"/>
+    <row r="24" spans="1:8" ht="15.75" customHeight="1"/>
+    <row r="25" spans="1:8" ht="15.75" customHeight="1"/>
+    <row r="26" spans="1:8" ht="15.75" customHeight="1"/>
+    <row r="27" spans="1:8" ht="15.75" customHeight="1"/>
+    <row r="28" spans="1:8" ht="15.75" customHeight="1"/>
+    <row r="29" spans="1:8" ht="15.75" customHeight="1"/>
+    <row r="30" spans="1:8" ht="15.75" customHeight="1"/>
+    <row r="31" spans="1:8" ht="15.75" customHeight="1"/>
+    <row r="32" spans="1:8" ht="15.75" customHeight="1"/>
     <row r="33" ht="15.75" customHeight="1"/>
     <row r="34" ht="15.75" customHeight="1"/>
     <row r="35" ht="15.75" customHeight="1"/>
@@ -2009,349 +2114,345 @@
     <row r="990" ht="15.75" customHeight="1"/>
     <row r="991" ht="15.75" customHeight="1"/>
   </sheetData>
-  <printOptions/>
-  <pageMargins bottom="0.787401575" footer="0.0" header="0.0" left="0.511811024" right="0.511811024" top="0.787401575"/>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-  <sheetPr>
-    <pageSetUpPr/>
-  </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:I1000"/>
+  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="3.0"/>
-    <col customWidth="1" min="2" max="2" width="11.0"/>
-    <col customWidth="1" min="3" max="3" width="13.63"/>
-    <col customWidth="1" min="4" max="4" width="45.13"/>
-    <col customWidth="1" min="5" max="5" width="14.38"/>
-    <col customWidth="1" min="6" max="6" width="14.63"/>
-    <col customWidth="1" min="7" max="7" width="14.0"/>
-    <col customWidth="1" min="8" max="8" width="35.38"/>
-    <col customWidth="1" min="9" max="9" width="11.13"/>
-    <col customWidth="1" min="10" max="26" width="8.63"/>
+    <col min="1" max="1" width="3" customWidth="1"/>
+    <col min="2" max="2" width="11" customWidth="1"/>
+    <col min="3" max="3" width="13.5703125" customWidth="1"/>
+    <col min="4" max="4" width="45.140625" customWidth="1"/>
+    <col min="5" max="5" width="14.42578125" customWidth="1"/>
+    <col min="6" max="6" width="14.5703125" customWidth="1"/>
+    <col min="7" max="7" width="14" customWidth="1"/>
+    <col min="8" max="8" width="35.42578125" customWidth="1"/>
+    <col min="9" max="9" width="11.140625" customWidth="1"/>
+    <col min="10" max="26" width="8.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:9">
       <c r="A1" s="1" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="2">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
       <c r="A2" s="1">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="B2" s="1">
-        <v>6803589.0</v>
+        <v>6803589</v>
       </c>
       <c r="C2" s="4">
-        <v>45950.0</v>
+        <v>45950</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="E2" s="1">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="G2" s="1">
         <v>20.2</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="I2" s="1">
-        <v>111.0</v>
-      </c>
-    </row>
-    <row r="3">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9">
       <c r="A3" s="1">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="B3" s="1">
-        <v>6398174.0</v>
+        <v>6398174</v>
       </c>
       <c r="C3" s="4">
-        <v>45953.0</v>
+        <v>45953</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="E3" s="1">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="G3" s="1">
-        <v>8.2</v>
+        <v>8.1999999999999993</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="I3" s="1">
-        <v>120.0</v>
-      </c>
-    </row>
-    <row r="4">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
       <c r="A4" s="1">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="B4" s="1">
-        <v>4415082.0</v>
+        <v>4415082</v>
       </c>
       <c r="C4" s="4">
-        <v>45945.0</v>
+        <v>45945</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="E4" s="1">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="G4" s="1">
         <v>2.5</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="I4" s="1">
-        <v>113.0</v>
-      </c>
-    </row>
-    <row r="5">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
       <c r="A5" s="1">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="B5" s="1">
-        <v>8154993.0</v>
+        <v>8154993</v>
       </c>
       <c r="C5" s="4">
-        <v>45940.0</v>
+        <v>45940</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="E5" s="1">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="G5" s="1">
         <v>0.6</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="I5" s="1">
-        <v>106.0</v>
-      </c>
-    </row>
-    <row r="6">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
       <c r="A6" s="1">
-        <v>7.0</v>
+        <v>7</v>
       </c>
       <c r="B6" s="1">
-        <v>6803204.0</v>
+        <v>6803204</v>
       </c>
       <c r="C6" s="4">
-        <v>46011.0</v>
+        <v>46011</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="E6" s="1">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="G6" s="1">
         <v>8.5</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="I6" s="1">
-        <v>122.0</v>
-      </c>
-    </row>
-    <row r="7">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9">
       <c r="A7" s="1">
-        <v>8.0</v>
+        <v>8</v>
       </c>
       <c r="B7" s="1">
-        <v>6398324.0</v>
+        <v>6398324</v>
       </c>
       <c r="C7" s="4">
-        <v>46014.0</v>
+        <v>46014</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="E7" s="1">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="G7" s="1">
-        <v>10.0</v>
+        <v>10</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="I7" s="1">
-        <v>125.0</v>
-      </c>
-    </row>
-    <row r="8">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9">
       <c r="A8" s="1">
-        <v>9.0</v>
+        <v>9</v>
       </c>
       <c r="B8" s="1">
-        <v>6338324.0</v>
+        <v>6338324</v>
       </c>
       <c r="C8" s="4">
-        <v>46018.0</v>
+        <v>46018</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="E8" s="1">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="G8" s="1">
-        <v>7.0</v>
+        <v>7</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="I8" s="1">
-        <v>125.0</v>
-      </c>
-    </row>
-    <row r="9">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9">
       <c r="A9" s="1">
-        <v>10.0</v>
+        <v>10</v>
       </c>
       <c r="B9" s="1">
-        <v>6975974.0</v>
+        <v>6975974</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="E9" s="1">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="G9" s="1">
-        <v>9.0</v>
+        <v>9</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="I9" s="1">
-        <v>125.0</v>
-      </c>
-    </row>
-    <row r="10">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9">
       <c r="A10" s="1">
-        <v>11.0</v>
+        <v>11</v>
       </c>
       <c r="B10" s="1">
-        <v>3215974.0</v>
+        <v>3215974</v>
       </c>
       <c r="C10" s="4">
-        <v>45993.0</v>
+        <v>45993</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="E10" s="1">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="G10" s="1">
-        <v>12.0</v>
+        <v>12</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="I10" s="1">
-        <v>125.0</v>
-      </c>
-    </row>
-    <row r="11">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9">
       <c r="A11" s="1">
-        <v>12.0</v>
+        <v>12</v>
       </c>
       <c r="B11" s="1">
-        <v>3288874.0</v>
+        <v>3288874</v>
       </c>
       <c r="C11" s="4">
-        <v>45997.0</v>
+        <v>45997</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="E11" s="1">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="G11" s="1">
         <v>5.5</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="I11" s="1">
-        <v>124.0</v>
+        <v>124</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -3335,627 +3436,623 @@
     <row r="999" ht="15.75" customHeight="1"/>
     <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
-  <printOptions/>
-  <pageMargins bottom="0.787401575" footer="0.0" header="0.0" left="0.511811024" right="0.511811024" top="0.787401575"/>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-  <sheetPr>
-    <pageSetUpPr/>
-  </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:C1000"/>
+  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="1" max="26" width="8.63"/>
+    <col min="1" max="26" width="8.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="2">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
       <c r="A2" s="1">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="B2" s="1">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="C2" s="1">
-        <v>6803589.0</v>
-      </c>
-    </row>
-    <row r="3">
+        <v>6803589</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
       <c r="A3" s="1">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="B3" s="1">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="C3" s="1">
-        <v>8154993.0</v>
-      </c>
-    </row>
-    <row r="4">
+        <v>8154993</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
       <c r="A4" s="1">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="B4" s="1">
-        <v>6.0</v>
+        <v>6</v>
       </c>
       <c r="C4" s="1">
-        <v>4415082.0</v>
-      </c>
-    </row>
-    <row r="5">
+        <v>4415082</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
       <c r="A5" s="1">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="B5" s="1">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="C5" s="1">
-        <v>6803589.0</v>
-      </c>
-    </row>
-    <row r="6">
+        <v>6803589</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
       <c r="A6" s="1">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="B6" s="1">
-        <v>15.0</v>
+        <v>15</v>
       </c>
       <c r="C6" s="1">
-        <v>8154993.0</v>
-      </c>
-    </row>
-    <row r="7">
+        <v>8154993</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
       <c r="A7" s="1">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="B7" s="1">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="C7" s="1">
-        <v>3215974.0</v>
-      </c>
-    </row>
-    <row r="8">
+        <v>3215974</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
       <c r="A8" s="1">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="B8" s="1">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="C8" s="1">
-        <v>6975974.0</v>
-      </c>
-    </row>
-    <row r="9">
+        <v>6975974</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
       <c r="A9" s="1">
-        <v>5.0</v>
+        <v>5</v>
       </c>
       <c r="B9" s="1">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="C9" s="1">
-        <v>6803589.0</v>
-      </c>
-    </row>
-    <row r="10">
+        <v>6803589</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
       <c r="A10" s="1">
-        <v>6.0</v>
+        <v>6</v>
       </c>
       <c r="B10" s="1">
-        <v>200.0</v>
+        <v>200</v>
       </c>
       <c r="C10" s="1">
-        <v>6803589.0</v>
-      </c>
-    </row>
-    <row r="11">
+        <v>6803589</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3">
       <c r="A11" s="1">
-        <v>8.0</v>
+        <v>8</v>
       </c>
       <c r="B11" s="1">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="C11" s="1">
-        <v>6803589.0</v>
-      </c>
-    </row>
-    <row r="12">
+        <v>6803589</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3">
       <c r="A12" s="1">
-        <v>10.0</v>
+        <v>10</v>
       </c>
       <c r="B12" s="1">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="C12" s="1">
-        <v>4415082.0</v>
-      </c>
-    </row>
-    <row r="13">
+        <v>4415082</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3">
       <c r="A13" s="1">
-        <v>10.0</v>
+        <v>10</v>
       </c>
       <c r="B13" s="1">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="C13" s="1">
-        <v>6803204.0</v>
-      </c>
-    </row>
-    <row r="14">
+        <v>6803204</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3">
       <c r="A14" s="1">
-        <v>10.0</v>
+        <v>10</v>
       </c>
       <c r="B14" s="1">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="C14" s="1">
-        <v>6803589.0</v>
-      </c>
-    </row>
-    <row r="15">
+        <v>6803589</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3">
       <c r="A15" s="1">
-        <v>10.0</v>
+        <v>10</v>
       </c>
       <c r="B15" s="1">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="C15" s="1">
-        <v>8154993.0</v>
-      </c>
-    </row>
-    <row r="16">
+        <v>8154993</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3">
       <c r="A16" s="1">
-        <v>11.0</v>
+        <v>11</v>
       </c>
       <c r="B16" s="1">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="C16" s="1">
-        <v>6803589.0</v>
-      </c>
-    </row>
-    <row r="17">
+        <v>6803589</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3">
       <c r="A17" s="1">
-        <v>12.0</v>
+        <v>12</v>
       </c>
       <c r="B17" s="1">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="C17" s="1">
-        <v>6803589.0</v>
-      </c>
-    </row>
-    <row r="18">
+        <v>6803589</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3">
       <c r="A18" s="1">
-        <v>12.0</v>
+        <v>12</v>
       </c>
       <c r="B18" s="1">
-        <v>200.0</v>
+        <v>200</v>
       </c>
       <c r="C18" s="1">
-        <v>8154993.0</v>
-      </c>
-    </row>
-    <row r="19">
+        <v>8154993</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3">
       <c r="A19" s="1">
-        <v>14.0</v>
+        <v>14</v>
       </c>
       <c r="B19" s="1">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="C19" s="1">
-        <v>6803589.0</v>
-      </c>
-    </row>
-    <row r="20">
+        <v>6803589</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3">
       <c r="A20" s="1">
-        <v>16.0</v>
+        <v>16</v>
       </c>
       <c r="B20" s="1">
-        <v>5.0</v>
+        <v>5</v>
       </c>
       <c r="C20" s="1">
-        <v>6338324.0</v>
-      </c>
-    </row>
-    <row r="21" ht="15.75" customHeight="1">
+        <v>6338324</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" ht="15.75" customHeight="1">
       <c r="A21" s="1">
-        <v>16.0</v>
+        <v>16</v>
       </c>
       <c r="B21" s="1">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="C21" s="1">
-        <v>6803589.0</v>
-      </c>
-    </row>
-    <row r="22" ht="15.75" customHeight="1">
+        <v>6803589</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" ht="15.75" customHeight="1">
       <c r="A22" s="1">
-        <v>17.0</v>
+        <v>17</v>
       </c>
       <c r="B22" s="1">
-        <v>5.0</v>
+        <v>5</v>
       </c>
       <c r="C22" s="1">
-        <v>6338324.0</v>
-      </c>
-    </row>
-    <row r="23" ht="15.75" customHeight="1">
+        <v>6338324</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" ht="15.75" customHeight="1">
       <c r="A23" s="1">
-        <v>17.0</v>
+        <v>17</v>
       </c>
       <c r="B23" s="1">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="C23" s="1">
-        <v>6803589.0</v>
-      </c>
-    </row>
-    <row r="24" ht="15.75" customHeight="1">
+        <v>6803589</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" ht="15.75" customHeight="1">
       <c r="A24" s="1">
-        <v>18.0</v>
+        <v>18</v>
       </c>
       <c r="B24" s="1">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="C24" s="1">
-        <v>6803589.0</v>
-      </c>
-    </row>
-    <row r="25" ht="15.75" customHeight="1">
+        <v>6803589</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" ht="15.75" customHeight="1">
       <c r="A25" s="1">
-        <v>19.0</v>
+        <v>19</v>
       </c>
       <c r="B25" s="1">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="C25" s="1">
-        <v>6803589.0</v>
-      </c>
-    </row>
-    <row r="26" ht="15.75" customHeight="1">
+        <v>6803589</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" ht="15.75" customHeight="1">
       <c r="A26" s="1">
-        <v>20.0</v>
+        <v>20</v>
       </c>
       <c r="B26" s="1">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="C26" s="1">
-        <v>3215974.0</v>
-      </c>
-    </row>
-    <row r="27" ht="15.75" customHeight="1">
+        <v>3215974</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" ht="15.75" customHeight="1">
       <c r="A27" s="1">
-        <v>20.0</v>
+        <v>20</v>
       </c>
       <c r="B27" s="1">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="C27" s="1">
-        <v>3288874.0</v>
-      </c>
-    </row>
-    <row r="28" ht="15.75" customHeight="1">
+        <v>3288874</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" ht="15.75" customHeight="1">
       <c r="A28" s="1">
-        <v>20.0</v>
+        <v>20</v>
       </c>
       <c r="B28" s="1">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="C28" s="1">
-        <v>6975974.0</v>
-      </c>
-    </row>
-    <row r="29" ht="15.75" customHeight="1">
+        <v>6975974</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" ht="15.75" customHeight="1">
       <c r="A29" s="1">
-        <v>21.0</v>
+        <v>21</v>
       </c>
       <c r="B29" s="1">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="C29" s="1">
-        <v>4415082.0</v>
-      </c>
-    </row>
-    <row r="30" ht="15.75" customHeight="1">
+        <v>4415082</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" ht="15.75" customHeight="1">
       <c r="A30" s="1">
-        <v>22.0</v>
+        <v>22</v>
       </c>
       <c r="B30" s="1">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="C30" s="1">
-        <v>3215974.0</v>
-      </c>
-    </row>
-    <row r="31" ht="15.75" customHeight="1">
+        <v>3215974</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" ht="15.75" customHeight="1">
       <c r="A31" s="1">
-        <v>22.0</v>
+        <v>22</v>
       </c>
       <c r="B31" s="1">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="C31" s="1">
-        <v>3288874.0</v>
-      </c>
-    </row>
-    <row r="32" ht="15.75" customHeight="1">
+        <v>3288874</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" ht="15.75" customHeight="1">
       <c r="A32" s="1">
-        <v>22.0</v>
+        <v>22</v>
       </c>
       <c r="B32" s="1">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="C32" s="1">
-        <v>6975974.0</v>
-      </c>
-    </row>
-    <row r="33" ht="15.75" customHeight="1">
+        <v>6975974</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" ht="15.75" customHeight="1">
       <c r="A33" s="1">
-        <v>23.0</v>
+        <v>23</v>
       </c>
       <c r="B33" s="1">
-        <v>25.0</v>
+        <v>25</v>
       </c>
       <c r="C33" s="1">
-        <v>6803204.0</v>
-      </c>
-    </row>
-    <row r="34" ht="15.75" customHeight="1">
+        <v>6803204</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" ht="15.75" customHeight="1">
       <c r="A34" s="1">
-        <v>24.0</v>
+        <v>24</v>
       </c>
       <c r="B34" s="1">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="C34" s="1">
-        <v>4415082.0</v>
-      </c>
-    </row>
-    <row r="35" ht="15.75" customHeight="1">
+        <v>4415082</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" ht="15.75" customHeight="1">
       <c r="A35" s="1">
-        <v>25.0</v>
+        <v>25</v>
       </c>
       <c r="B35" s="1">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="C35" s="1">
-        <v>3288874.0</v>
-      </c>
-    </row>
-    <row r="36" ht="15.75" customHeight="1">
+        <v>3288874</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" ht="15.75" customHeight="1">
       <c r="A36" s="1">
-        <v>25.0</v>
+        <v>25</v>
       </c>
       <c r="B36" s="1">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="C36" s="1">
-        <v>6398174.0</v>
-      </c>
-    </row>
-    <row r="37" ht="15.75" customHeight="1">
+        <v>6398174</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" ht="15.75" customHeight="1">
       <c r="A37" s="1">
-        <v>25.0</v>
+        <v>25</v>
       </c>
       <c r="B37" s="1">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="C37" s="1">
-        <v>6803589.0</v>
-      </c>
-    </row>
-    <row r="38" ht="15.75" customHeight="1">
+        <v>6803589</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" ht="15.75" customHeight="1">
       <c r="A38" s="1">
-        <v>26.0</v>
+        <v>26</v>
       </c>
       <c r="B38" s="1">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="C38" s="1">
-        <v>6803589.0</v>
-      </c>
-    </row>
-    <row r="39" ht="15.75" customHeight="1">
+        <v>6803589</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" ht="15.75" customHeight="1">
       <c r="A39" s="1">
-        <v>27.0</v>
+        <v>27</v>
       </c>
       <c r="B39" s="1">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="C39" s="1">
-        <v>6803589.0</v>
-      </c>
-    </row>
-    <row r="40" ht="15.75" customHeight="1">
+        <v>6803589</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" ht="15.75" customHeight="1">
       <c r="A40" s="1">
-        <v>28.0</v>
+        <v>28</v>
       </c>
       <c r="B40" s="1">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="C40" s="1">
-        <v>4415082.0</v>
-      </c>
-    </row>
-    <row r="41" ht="15.75" customHeight="1">
+        <v>4415082</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" ht="15.75" customHeight="1">
       <c r="A41" s="1">
-        <v>28.0</v>
+        <v>28</v>
       </c>
       <c r="B41" s="1">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="C41" s="1">
-        <v>6398174.0</v>
-      </c>
-    </row>
-    <row r="42" ht="15.75" customHeight="1">
+        <v>6398174</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" ht="15.75" customHeight="1">
       <c r="A42" s="1">
-        <v>28.0</v>
+        <v>28</v>
       </c>
       <c r="B42" s="1">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="C42" s="1">
-        <v>6803589.0</v>
-      </c>
-    </row>
-    <row r="43" ht="15.75" customHeight="1">
+        <v>6803589</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" ht="15.75" customHeight="1">
       <c r="A43" s="1">
-        <v>28.0</v>
+        <v>28</v>
       </c>
       <c r="B43" s="1">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="C43" s="1">
-        <v>8154993.0</v>
-      </c>
-    </row>
-    <row r="44" ht="15.75" customHeight="1">
+        <v>8154993</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" ht="15.75" customHeight="1">
       <c r="A44" s="1">
-        <v>29.0</v>
+        <v>29</v>
       </c>
       <c r="B44" s="1">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="C44" s="1">
-        <v>6803589.0</v>
-      </c>
-    </row>
-    <row r="45" ht="15.75" customHeight="1">
+        <v>6803589</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" ht="15.75" customHeight="1">
       <c r="A45" s="1">
-        <v>30.0</v>
+        <v>30</v>
       </c>
       <c r="B45" s="1">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="C45" s="1">
-        <v>6803589.0</v>
-      </c>
-    </row>
-    <row r="46" ht="15.75" customHeight="1">
+        <v>6803589</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" ht="15.75" customHeight="1">
       <c r="A46" s="1">
-        <v>31.0</v>
+        <v>31</v>
       </c>
       <c r="B46" s="1">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="C46" s="1">
-        <v>4415082.0</v>
-      </c>
-    </row>
-    <row r="47" ht="15.75" customHeight="1">
+        <v>4415082</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" ht="15.75" customHeight="1">
       <c r="A47" s="1">
-        <v>32.0</v>
+        <v>32</v>
       </c>
       <c r="B47" s="1">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="C47" s="1">
-        <v>4415082.0</v>
-      </c>
-    </row>
-    <row r="48" ht="15.75" customHeight="1">
+        <v>4415082</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" ht="15.75" customHeight="1">
       <c r="A48" s="1">
-        <v>32.0</v>
+        <v>32</v>
       </c>
       <c r="B48" s="1">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="C48" s="1">
-        <v>6803589.0</v>
-      </c>
-    </row>
-    <row r="49" ht="15.75" customHeight="1">
+        <v>6803589</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" ht="15.75" customHeight="1">
       <c r="A49" s="1">
-        <v>32.0</v>
+        <v>32</v>
       </c>
       <c r="B49" s="1">
-        <v>10.0</v>
+        <v>10</v>
       </c>
       <c r="C49" s="1">
-        <v>8154993.0</v>
-      </c>
-    </row>
-    <row r="50" ht="15.75" customHeight="1">
+        <v>8154993</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" ht="15.75" customHeight="1">
       <c r="A50" s="1">
-        <v>33.0</v>
+        <v>33</v>
       </c>
       <c r="B50" s="1">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="C50" s="1">
-        <v>4415082.0</v>
-      </c>
-    </row>
-    <row r="51" ht="15.75" customHeight="1">
+        <v>4415082</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" ht="15.75" customHeight="1">
       <c r="A51" s="1">
-        <v>33.0</v>
+        <v>33</v>
       </c>
       <c r="B51" s="1">
-        <v>5.0</v>
+        <v>5</v>
       </c>
       <c r="C51" s="1">
-        <v>8154993.0</v>
-      </c>
-    </row>
-    <row r="52" ht="15.75" customHeight="1">
+        <v>8154993</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" ht="15.75" customHeight="1">
       <c r="A52" s="1">
-        <v>34.0</v>
+        <v>34</v>
       </c>
       <c r="B52" s="1">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="C52" s="1">
-        <v>6398174.0</v>
-      </c>
-    </row>
-    <row r="53" ht="15.75" customHeight="1">
+        <v>6398174</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" ht="15.75" customHeight="1">
       <c r="A53" s="1">
-        <v>34.0</v>
+        <v>34</v>
       </c>
       <c r="B53" s="1">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="C53" s="1">
-        <v>6803204.0</v>
-      </c>
-    </row>
-    <row r="54" ht="15.75" customHeight="1">
+        <v>6803204</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" ht="15.75" customHeight="1">
       <c r="A54" s="1">
-        <v>34.0</v>
+        <v>34</v>
       </c>
       <c r="B54" s="1">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="C54" s="1">
-        <v>6803589.0</v>
-      </c>
-    </row>
-    <row r="55" ht="15.75" customHeight="1"/>
-    <row r="56" ht="15.75" customHeight="1"/>
-    <row r="57" ht="15.75" customHeight="1"/>
-    <row r="58" ht="15.75" customHeight="1"/>
-    <row r="59" ht="15.75" customHeight="1"/>
-    <row r="60" ht="15.75" customHeight="1"/>
-    <row r="61" ht="15.75" customHeight="1"/>
-    <row r="62" ht="15.75" customHeight="1"/>
-    <row r="63" ht="15.75" customHeight="1"/>
-    <row r="64" ht="15.75" customHeight="1"/>
+        <v>6803589</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" ht="15.75" customHeight="1"/>
+    <row r="56" spans="1:3" ht="15.75" customHeight="1"/>
+    <row r="57" spans="1:3" ht="15.75" customHeight="1"/>
+    <row r="58" spans="1:3" ht="15.75" customHeight="1"/>
+    <row r="59" spans="1:3" ht="15.75" customHeight="1"/>
+    <row r="60" spans="1:3" ht="15.75" customHeight="1"/>
+    <row r="61" spans="1:3" ht="15.75" customHeight="1"/>
+    <row r="62" spans="1:3" ht="15.75" customHeight="1"/>
+    <row r="63" spans="1:3" ht="15.75" customHeight="1"/>
+    <row r="64" spans="1:3" ht="15.75" customHeight="1"/>
     <row r="65" ht="15.75" customHeight="1"/>
     <row r="66" ht="15.75" customHeight="1"/>
     <row r="67" ht="15.75" customHeight="1"/>
@@ -4893,9 +4990,7 @@
     <row r="999" ht="15.75" customHeight="1"/>
     <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
-  <printOptions/>
-  <pageMargins bottom="0.787401575" footer="0.0" header="0.0" left="0.511811024" right="0.511811024" top="0.787401575"/>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>